<commit_message>
data: update Nam Dinh lottery results
</commit_message>
<xml_diff>
--- a/outputs/result_scraping/nam_dinh_results.xlsx
+++ b/outputs/result_scraping/nam_dinh_results.xlsx
@@ -6,7 +6,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nam Dinh Results" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Nam Dinh Results'!$A$1:$D$226</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Nam Dinh Results'!$A$1:$D$301</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Nam Dinh Results'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
@@ -1399,13 +1399,388 @@
         <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-11-12</t>
       </text>
     </comment>
+    <comment ref="A227" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-11-13</t>
+      </text>
+    </comment>
+    <comment ref="A228" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-11-14</t>
+      </text>
+    </comment>
+    <comment ref="A229" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-11-15</t>
+      </text>
+    </comment>
+    <comment ref="A230" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-11-16</t>
+      </text>
+    </comment>
+    <comment ref="A231" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-11-17</t>
+      </text>
+    </comment>
+    <comment ref="A232" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-11-18</t>
+      </text>
+    </comment>
+    <comment ref="A233" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-11-19</t>
+      </text>
+    </comment>
+    <comment ref="A234" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-11-20</t>
+      </text>
+    </comment>
+    <comment ref="A235" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-11-21</t>
+      </text>
+    </comment>
+    <comment ref="A236" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-11-22</t>
+      </text>
+    </comment>
+    <comment ref="A237" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-11-23</t>
+      </text>
+    </comment>
+    <comment ref="A238" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-11-24</t>
+      </text>
+    </comment>
+    <comment ref="A239" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-11-25</t>
+      </text>
+    </comment>
+    <comment ref="A240" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-11-26</t>
+      </text>
+    </comment>
+    <comment ref="A241" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-11-27</t>
+      </text>
+    </comment>
+    <comment ref="A242" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-11-28</t>
+      </text>
+    </comment>
+    <comment ref="A243" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-11-29</t>
+      </text>
+    </comment>
+    <comment ref="A244" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-11-30</t>
+      </text>
+    </comment>
+    <comment ref="A245" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-12-01</t>
+      </text>
+    </comment>
+    <comment ref="A246" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-12-02</t>
+      </text>
+    </comment>
+    <comment ref="A247" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-12-03</t>
+      </text>
+    </comment>
+    <comment ref="A248" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-12-04</t>
+      </text>
+    </comment>
+    <comment ref="A249" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-12-05</t>
+      </text>
+    </comment>
+    <comment ref="A250" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-12-06</t>
+      </text>
+    </comment>
+    <comment ref="A251" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-12-07</t>
+      </text>
+    </comment>
+    <comment ref="A252" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-12-08</t>
+      </text>
+    </comment>
+    <comment ref="A253" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-12-09</t>
+      </text>
+    </comment>
+    <comment ref="A254" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-12-10</t>
+      </text>
+    </comment>
+    <comment ref="A255" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-12-11</t>
+      </text>
+    </comment>
+    <comment ref="A256" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-12-12</t>
+      </text>
+    </comment>
+    <comment ref="A257" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-12-13</t>
+      </text>
+    </comment>
+    <comment ref="A258" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-12-14</t>
+      </text>
+    </comment>
+    <comment ref="A259" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-12-15</t>
+      </text>
+    </comment>
+    <comment ref="A260" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-12-16</t>
+      </text>
+    </comment>
+    <comment ref="A261" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-12-17</t>
+      </text>
+    </comment>
+    <comment ref="A262" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-12-18</t>
+      </text>
+    </comment>
+    <comment ref="A263" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-12-19</t>
+      </text>
+    </comment>
+    <comment ref="A264" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-12-20</t>
+      </text>
+    </comment>
+    <comment ref="A265" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-12-21</t>
+      </text>
+    </comment>
+    <comment ref="A266" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-12-22</t>
+      </text>
+    </comment>
+    <comment ref="A267" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-12-23</t>
+      </text>
+    </comment>
+    <comment ref="A268" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-12-24</t>
+      </text>
+    </comment>
+    <comment ref="A269" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-12-25</t>
+      </text>
+    </comment>
+    <comment ref="A270" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-12-26</t>
+      </text>
+    </comment>
+    <comment ref="A271" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-12-27</t>
+      </text>
+    </comment>
+    <comment ref="A272" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-12-28</t>
+      </text>
+    </comment>
+    <comment ref="A273" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-12-29</t>
+      </text>
+    </comment>
+    <comment ref="A274" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-12-30</t>
+      </text>
+    </comment>
+    <comment ref="A275" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2020-12-31</t>
+      </text>
+    </comment>
+    <comment ref="A276" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2021-01-01</t>
+      </text>
+    </comment>
+    <comment ref="A277" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2021-01-02</t>
+      </text>
+    </comment>
+    <comment ref="A278" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2021-01-03</t>
+      </text>
+    </comment>
+    <comment ref="A279" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2021-01-04</t>
+      </text>
+    </comment>
+    <comment ref="A280" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2021-01-05</t>
+      </text>
+    </comment>
+    <comment ref="A281" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2021-01-06</t>
+      </text>
+    </comment>
+    <comment ref="A282" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2021-01-07</t>
+      </text>
+    </comment>
+    <comment ref="A283" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2021-01-08</t>
+      </text>
+    </comment>
+    <comment ref="A284" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2021-01-09</t>
+      </text>
+    </comment>
+    <comment ref="A285" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2021-01-10</t>
+      </text>
+    </comment>
+    <comment ref="A286" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2021-01-11</t>
+      </text>
+    </comment>
+    <comment ref="A287" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2021-01-12</t>
+      </text>
+    </comment>
+    <comment ref="A288" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2021-01-13</t>
+      </text>
+    </comment>
+    <comment ref="A289" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2021-01-14</t>
+      </text>
+    </comment>
+    <comment ref="A290" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2021-01-15</t>
+      </text>
+    </comment>
+    <comment ref="A291" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2021-01-16</t>
+      </text>
+    </comment>
+    <comment ref="A292" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2021-01-17</t>
+      </text>
+    </comment>
+    <comment ref="A293" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2021-01-18</t>
+      </text>
+    </comment>
+    <comment ref="A294" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2021-01-19</t>
+      </text>
+    </comment>
+    <comment ref="A295" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2021-01-20</t>
+      </text>
+    </comment>
+    <comment ref="A296" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2021-01-21</t>
+      </text>
+    </comment>
+    <comment ref="A297" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2021-01-22</t>
+      </text>
+    </comment>
+    <comment ref="A298" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2021-01-23</t>
+      </text>
+    </comment>
+    <comment ref="A299" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2021-01-24</t>
+      </text>
+    </comment>
+    <comment ref="A300" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2021-01-25</t>
+      </text>
+    </comment>
+    <comment ref="A301" authorId="0" shapeId="0">
+      <text>
+        <t>Official source: https://www.thinhnam.net.in/ket-qua-xo-so-mien-nam.php?ngay=2021-01-26</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="NamDinhResults" displayName="NamDinhResults" ref="A1:D226" headerRowCount="1">
-  <autoFilter ref="A1:D226"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="NamDinhResults" displayName="NamDinhResults" ref="A1:D301" headerRowCount="1">
+  <autoFilter ref="A1:D301"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Date"/>
     <tableColumn id="2" name="Grand Prize"/>
@@ -1613,7 +1988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D226"/>
+  <dimension ref="A1:D301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -5244,8 +5619,1208 @@
         <v/>
       </c>
     </row>
+    <row r="227" ht="20" customHeight="1">
+      <c r="A227" s="29" t="n">
+        <v>44148</v>
+      </c>
+      <c r="B227" s="30" t="n">
+        <v>83132</v>
+      </c>
+      <c r="C227" s="30">
+        <f>MOD(B227,100)*1000+INT(B227/100)</f>
+        <v/>
+      </c>
+      <c r="D227" s="30">
+        <f>INT(B227/10000)*10000+MOD(B227,10)*1000+INT(MOD(B227,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="228" ht="20" customHeight="1">
+      <c r="A228" s="27" t="n">
+        <v>44149</v>
+      </c>
+      <c r="B228" s="28" t="n">
+        <v>91699</v>
+      </c>
+      <c r="C228" s="28">
+        <f>MOD(B228,100)*1000+INT(B228/100)</f>
+        <v/>
+      </c>
+      <c r="D228" s="28">
+        <f>INT(B228/10000)*10000+MOD(B228,10)*1000+INT(MOD(B228,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="229" ht="20" customHeight="1">
+      <c r="A229" s="29" t="n">
+        <v>44150</v>
+      </c>
+      <c r="B229" s="30" t="n">
+        <v>59575</v>
+      </c>
+      <c r="C229" s="30">
+        <f>MOD(B229,100)*1000+INT(B229/100)</f>
+        <v/>
+      </c>
+      <c r="D229" s="30">
+        <f>INT(B229/10000)*10000+MOD(B229,10)*1000+INT(MOD(B229,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="230" ht="20" customHeight="1">
+      <c r="A230" s="27" t="n">
+        <v>44151</v>
+      </c>
+      <c r="B230" s="28" t="n">
+        <v>87103</v>
+      </c>
+      <c r="C230" s="28">
+        <f>MOD(B230,100)*1000+INT(B230/100)</f>
+        <v/>
+      </c>
+      <c r="D230" s="28">
+        <f>INT(B230/10000)*10000+MOD(B230,10)*1000+INT(MOD(B230,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="231" ht="20" customHeight="1">
+      <c r="A231" s="29" t="n">
+        <v>44152</v>
+      </c>
+      <c r="B231" s="30" t="n">
+        <v>55515</v>
+      </c>
+      <c r="C231" s="30">
+        <f>MOD(B231,100)*1000+INT(B231/100)</f>
+        <v/>
+      </c>
+      <c r="D231" s="30">
+        <f>INT(B231/10000)*10000+MOD(B231,10)*1000+INT(MOD(B231,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="232" ht="20" customHeight="1">
+      <c r="A232" s="27" t="n">
+        <v>44153</v>
+      </c>
+      <c r="B232" s="28" t="n">
+        <v>26233</v>
+      </c>
+      <c r="C232" s="28">
+        <f>MOD(B232,100)*1000+INT(B232/100)</f>
+        <v/>
+      </c>
+      <c r="D232" s="28">
+        <f>INT(B232/10000)*10000+MOD(B232,10)*1000+INT(MOD(B232,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="233" ht="20" customHeight="1">
+      <c r="A233" s="29" t="n">
+        <v>44154</v>
+      </c>
+      <c r="B233" s="30" t="n">
+        <v>39763</v>
+      </c>
+      <c r="C233" s="30">
+        <f>MOD(B233,100)*1000+INT(B233/100)</f>
+        <v/>
+      </c>
+      <c r="D233" s="30">
+        <f>INT(B233/10000)*10000+MOD(B233,10)*1000+INT(MOD(B233,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="234" ht="20" customHeight="1">
+      <c r="A234" s="27" t="n">
+        <v>44155</v>
+      </c>
+      <c r="B234" s="28" t="n">
+        <v>71137</v>
+      </c>
+      <c r="C234" s="28">
+        <f>MOD(B234,100)*1000+INT(B234/100)</f>
+        <v/>
+      </c>
+      <c r="D234" s="28">
+        <f>INT(B234/10000)*10000+MOD(B234,10)*1000+INT(MOD(B234,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="235" ht="20" customHeight="1">
+      <c r="A235" s="29" t="n">
+        <v>44156</v>
+      </c>
+      <c r="B235" s="30" t="n">
+        <v>33507</v>
+      </c>
+      <c r="C235" s="30">
+        <f>MOD(B235,100)*1000+INT(B235/100)</f>
+        <v/>
+      </c>
+      <c r="D235" s="30">
+        <f>INT(B235/10000)*10000+MOD(B235,10)*1000+INT(MOD(B235,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="236" ht="20" customHeight="1">
+      <c r="A236" s="27" t="n">
+        <v>44157</v>
+      </c>
+      <c r="B236" s="28" t="n">
+        <v>93037</v>
+      </c>
+      <c r="C236" s="28">
+        <f>MOD(B236,100)*1000+INT(B236/100)</f>
+        <v/>
+      </c>
+      <c r="D236" s="28">
+        <f>INT(B236/10000)*10000+MOD(B236,10)*1000+INT(MOD(B236,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="237" ht="20" customHeight="1">
+      <c r="A237" s="29" t="n">
+        <v>44158</v>
+      </c>
+      <c r="B237" s="30" t="n">
+        <v>97806</v>
+      </c>
+      <c r="C237" s="30">
+        <f>MOD(B237,100)*1000+INT(B237/100)</f>
+        <v/>
+      </c>
+      <c r="D237" s="30">
+        <f>INT(B237/10000)*10000+MOD(B237,10)*1000+INT(MOD(B237,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="238" ht="20" customHeight="1">
+      <c r="A238" s="27" t="n">
+        <v>44159</v>
+      </c>
+      <c r="B238" s="28" t="n">
+        <v>38061</v>
+      </c>
+      <c r="C238" s="28">
+        <f>MOD(B238,100)*1000+INT(B238/100)</f>
+        <v/>
+      </c>
+      <c r="D238" s="28">
+        <f>INT(B238/10000)*10000+MOD(B238,10)*1000+INT(MOD(B238,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="239" ht="20" customHeight="1">
+      <c r="A239" s="29" t="n">
+        <v>44160</v>
+      </c>
+      <c r="B239" s="30" t="n">
+        <v>31010</v>
+      </c>
+      <c r="C239" s="30">
+        <f>MOD(B239,100)*1000+INT(B239/100)</f>
+        <v/>
+      </c>
+      <c r="D239" s="30">
+        <f>INT(B239/10000)*10000+MOD(B239,10)*1000+INT(MOD(B239,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="240" ht="20" customHeight="1">
+      <c r="A240" s="27" t="n">
+        <v>44161</v>
+      </c>
+      <c r="B240" s="28" t="n">
+        <v>73276</v>
+      </c>
+      <c r="C240" s="28">
+        <f>MOD(B240,100)*1000+INT(B240/100)</f>
+        <v/>
+      </c>
+      <c r="D240" s="28">
+        <f>INT(B240/10000)*10000+MOD(B240,10)*1000+INT(MOD(B240,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="241" ht="20" customHeight="1">
+      <c r="A241" s="29" t="n">
+        <v>44162</v>
+      </c>
+      <c r="B241" s="30" t="n">
+        <v>57304</v>
+      </c>
+      <c r="C241" s="30">
+        <f>MOD(B241,100)*1000+INT(B241/100)</f>
+        <v/>
+      </c>
+      <c r="D241" s="30">
+        <f>INT(B241/10000)*10000+MOD(B241,10)*1000+INT(MOD(B241,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="242" ht="20" customHeight="1">
+      <c r="A242" s="27" t="n">
+        <v>44163</v>
+      </c>
+      <c r="B242" s="28" t="n">
+        <v>86187</v>
+      </c>
+      <c r="C242" s="28">
+        <f>MOD(B242,100)*1000+INT(B242/100)</f>
+        <v/>
+      </c>
+      <c r="D242" s="28">
+        <f>INT(B242/10000)*10000+MOD(B242,10)*1000+INT(MOD(B242,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="243" ht="20" customHeight="1">
+      <c r="A243" s="29" t="n">
+        <v>44164</v>
+      </c>
+      <c r="B243" s="30" t="n">
+        <v>21764</v>
+      </c>
+      <c r="C243" s="30">
+        <f>MOD(B243,100)*1000+INT(B243/100)</f>
+        <v/>
+      </c>
+      <c r="D243" s="30">
+        <f>INT(B243/10000)*10000+MOD(B243,10)*1000+INT(MOD(B243,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="244" ht="20" customHeight="1">
+      <c r="A244" s="27" t="n">
+        <v>44165</v>
+      </c>
+      <c r="B244" s="28" t="n">
+        <v>36392</v>
+      </c>
+      <c r="C244" s="28">
+        <f>MOD(B244,100)*1000+INT(B244/100)</f>
+        <v/>
+      </c>
+      <c r="D244" s="28">
+        <f>INT(B244/10000)*10000+MOD(B244,10)*1000+INT(MOD(B244,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="245" ht="20" customHeight="1">
+      <c r="A245" s="29" t="n">
+        <v>44166</v>
+      </c>
+      <c r="B245" s="30" t="n">
+        <v>60931</v>
+      </c>
+      <c r="C245" s="30">
+        <f>MOD(B245,100)*1000+INT(B245/100)</f>
+        <v/>
+      </c>
+      <c r="D245" s="30">
+        <f>INT(B245/10000)*10000+MOD(B245,10)*1000+INT(MOD(B245,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="246" ht="20" customHeight="1">
+      <c r="A246" s="27" t="n">
+        <v>44167</v>
+      </c>
+      <c r="B246" s="28" t="n">
+        <v>49290</v>
+      </c>
+      <c r="C246" s="28">
+        <f>MOD(B246,100)*1000+INT(B246/100)</f>
+        <v/>
+      </c>
+      <c r="D246" s="28">
+        <f>INT(B246/10000)*10000+MOD(B246,10)*1000+INT(MOD(B246,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="247" ht="20" customHeight="1">
+      <c r="A247" s="29" t="n">
+        <v>44168</v>
+      </c>
+      <c r="B247" s="30" t="n">
+        <v>85728</v>
+      </c>
+      <c r="C247" s="30">
+        <f>MOD(B247,100)*1000+INT(B247/100)</f>
+        <v/>
+      </c>
+      <c r="D247" s="30">
+        <f>INT(B247/10000)*10000+MOD(B247,10)*1000+INT(MOD(B247,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="248" ht="20" customHeight="1">
+      <c r="A248" s="27" t="n">
+        <v>44169</v>
+      </c>
+      <c r="B248" s="28" t="n">
+        <v>55538</v>
+      </c>
+      <c r="C248" s="28">
+        <f>MOD(B248,100)*1000+INT(B248/100)</f>
+        <v/>
+      </c>
+      <c r="D248" s="28">
+        <f>INT(B248/10000)*10000+MOD(B248,10)*1000+INT(MOD(B248,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="249" ht="20" customHeight="1">
+      <c r="A249" s="29" t="n">
+        <v>44170</v>
+      </c>
+      <c r="B249" s="30" t="n">
+        <v>74361</v>
+      </c>
+      <c r="C249" s="30">
+        <f>MOD(B249,100)*1000+INT(B249/100)</f>
+        <v/>
+      </c>
+      <c r="D249" s="30">
+        <f>INT(B249/10000)*10000+MOD(B249,10)*1000+INT(MOD(B249,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="250" ht="20" customHeight="1">
+      <c r="A250" s="27" t="n">
+        <v>44171</v>
+      </c>
+      <c r="B250" s="28" t="n">
+        <v>49576</v>
+      </c>
+      <c r="C250" s="28">
+        <f>MOD(B250,100)*1000+INT(B250/100)</f>
+        <v/>
+      </c>
+      <c r="D250" s="28">
+        <f>INT(B250/10000)*10000+MOD(B250,10)*1000+INT(MOD(B250,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="251" ht="20" customHeight="1">
+      <c r="A251" s="29" t="n">
+        <v>44172</v>
+      </c>
+      <c r="B251" s="30" t="n">
+        <v>59688</v>
+      </c>
+      <c r="C251" s="30">
+        <f>MOD(B251,100)*1000+INT(B251/100)</f>
+        <v/>
+      </c>
+      <c r="D251" s="30">
+        <f>INT(B251/10000)*10000+MOD(B251,10)*1000+INT(MOD(B251,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="252" ht="20" customHeight="1">
+      <c r="A252" s="27" t="n">
+        <v>44173</v>
+      </c>
+      <c r="B252" s="28" t="n">
+        <v>73170</v>
+      </c>
+      <c r="C252" s="28">
+        <f>MOD(B252,100)*1000+INT(B252/100)</f>
+        <v/>
+      </c>
+      <c r="D252" s="28">
+        <f>INT(B252/10000)*10000+MOD(B252,10)*1000+INT(MOD(B252,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="253" ht="20" customHeight="1">
+      <c r="A253" s="29" t="n">
+        <v>44174</v>
+      </c>
+      <c r="B253" s="30" t="n">
+        <v>28198</v>
+      </c>
+      <c r="C253" s="30">
+        <f>MOD(B253,100)*1000+INT(B253/100)</f>
+        <v/>
+      </c>
+      <c r="D253" s="30">
+        <f>INT(B253/10000)*10000+MOD(B253,10)*1000+INT(MOD(B253,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="254" ht="20" customHeight="1">
+      <c r="A254" s="27" t="n">
+        <v>44175</v>
+      </c>
+      <c r="B254" s="28" t="n">
+        <v>90283</v>
+      </c>
+      <c r="C254" s="28">
+        <f>MOD(B254,100)*1000+INT(B254/100)</f>
+        <v/>
+      </c>
+      <c r="D254" s="28">
+        <f>INT(B254/10000)*10000+MOD(B254,10)*1000+INT(MOD(B254,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="255" ht="20" customHeight="1">
+      <c r="A255" s="29" t="n">
+        <v>44176</v>
+      </c>
+      <c r="B255" s="30" t="n">
+        <v>13044</v>
+      </c>
+      <c r="C255" s="30">
+        <f>MOD(B255,100)*1000+INT(B255/100)</f>
+        <v/>
+      </c>
+      <c r="D255" s="30">
+        <f>INT(B255/10000)*10000+MOD(B255,10)*1000+INT(MOD(B255,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="256" ht="20" customHeight="1">
+      <c r="A256" s="27" t="n">
+        <v>44177</v>
+      </c>
+      <c r="B256" s="28" t="n">
+        <v>16476</v>
+      </c>
+      <c r="C256" s="28">
+        <f>MOD(B256,100)*1000+INT(B256/100)</f>
+        <v/>
+      </c>
+      <c r="D256" s="28">
+        <f>INT(B256/10000)*10000+MOD(B256,10)*1000+INT(MOD(B256,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="257" ht="20" customHeight="1">
+      <c r="A257" s="29" t="n">
+        <v>44178</v>
+      </c>
+      <c r="B257" s="30" t="n">
+        <v>96763</v>
+      </c>
+      <c r="C257" s="30">
+        <f>MOD(B257,100)*1000+INT(B257/100)</f>
+        <v/>
+      </c>
+      <c r="D257" s="30">
+        <f>INT(B257/10000)*10000+MOD(B257,10)*1000+INT(MOD(B257,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="258" ht="20" customHeight="1">
+      <c r="A258" s="27" t="n">
+        <v>44179</v>
+      </c>
+      <c r="B258" s="28" t="n">
+        <v>23417</v>
+      </c>
+      <c r="C258" s="28">
+        <f>MOD(B258,100)*1000+INT(B258/100)</f>
+        <v/>
+      </c>
+      <c r="D258" s="28">
+        <f>INT(B258/10000)*10000+MOD(B258,10)*1000+INT(MOD(B258,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="259" ht="20" customHeight="1">
+      <c r="A259" s="29" t="n">
+        <v>44180</v>
+      </c>
+      <c r="B259" s="30" t="n">
+        <v>31793</v>
+      </c>
+      <c r="C259" s="30">
+        <f>MOD(B259,100)*1000+INT(B259/100)</f>
+        <v/>
+      </c>
+      <c r="D259" s="30">
+        <f>INT(B259/10000)*10000+MOD(B259,10)*1000+INT(MOD(B259,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="260" ht="20" customHeight="1">
+      <c r="A260" s="27" t="n">
+        <v>44181</v>
+      </c>
+      <c r="B260" s="28" t="n">
+        <v>90053</v>
+      </c>
+      <c r="C260" s="28">
+        <f>MOD(B260,100)*1000+INT(B260/100)</f>
+        <v/>
+      </c>
+      <c r="D260" s="28">
+        <f>INT(B260/10000)*10000+MOD(B260,10)*1000+INT(MOD(B260,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="261" ht="20" customHeight="1">
+      <c r="A261" s="29" t="n">
+        <v>44182</v>
+      </c>
+      <c r="B261" s="30" t="n">
+        <v>32141</v>
+      </c>
+      <c r="C261" s="30">
+        <f>MOD(B261,100)*1000+INT(B261/100)</f>
+        <v/>
+      </c>
+      <c r="D261" s="30">
+        <f>INT(B261/10000)*10000+MOD(B261,10)*1000+INT(MOD(B261,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="262" ht="20" customHeight="1">
+      <c r="A262" s="27" t="n">
+        <v>44183</v>
+      </c>
+      <c r="B262" s="28" t="n">
+        <v>58173</v>
+      </c>
+      <c r="C262" s="28">
+        <f>MOD(B262,100)*1000+INT(B262/100)</f>
+        <v/>
+      </c>
+      <c r="D262" s="28">
+        <f>INT(B262/10000)*10000+MOD(B262,10)*1000+INT(MOD(B262,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="263" ht="20" customHeight="1">
+      <c r="A263" s="29" t="n">
+        <v>44184</v>
+      </c>
+      <c r="B263" s="30" t="n">
+        <v>94640</v>
+      </c>
+      <c r="C263" s="30">
+        <f>MOD(B263,100)*1000+INT(B263/100)</f>
+        <v/>
+      </c>
+      <c r="D263" s="30">
+        <f>INT(B263/10000)*10000+MOD(B263,10)*1000+INT(MOD(B263,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="264" ht="20" customHeight="1">
+      <c r="A264" s="27" t="n">
+        <v>44185</v>
+      </c>
+      <c r="B264" s="28" t="n">
+        <v>88153</v>
+      </c>
+      <c r="C264" s="28">
+        <f>MOD(B264,100)*1000+INT(B264/100)</f>
+        <v/>
+      </c>
+      <c r="D264" s="28">
+        <f>INT(B264/10000)*10000+MOD(B264,10)*1000+INT(MOD(B264,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="265" ht="20" customHeight="1">
+      <c r="A265" s="29" t="n">
+        <v>44186</v>
+      </c>
+      <c r="B265" s="30" t="n">
+        <v>15125</v>
+      </c>
+      <c r="C265" s="30">
+        <f>MOD(B265,100)*1000+INT(B265/100)</f>
+        <v/>
+      </c>
+      <c r="D265" s="30">
+        <f>INT(B265/10000)*10000+MOD(B265,10)*1000+INT(MOD(B265,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="266" ht="20" customHeight="1">
+      <c r="A266" s="27" t="n">
+        <v>44187</v>
+      </c>
+      <c r="B266" s="28" t="n">
+        <v>34971</v>
+      </c>
+      <c r="C266" s="28">
+        <f>MOD(B266,100)*1000+INT(B266/100)</f>
+        <v/>
+      </c>
+      <c r="D266" s="28">
+        <f>INT(B266/10000)*10000+MOD(B266,10)*1000+INT(MOD(B266,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="267" ht="20" customHeight="1">
+      <c r="A267" s="29" t="n">
+        <v>44188</v>
+      </c>
+      <c r="B267" s="30" t="n">
+        <v>68989</v>
+      </c>
+      <c r="C267" s="30">
+        <f>MOD(B267,100)*1000+INT(B267/100)</f>
+        <v/>
+      </c>
+      <c r="D267" s="30">
+        <f>INT(B267/10000)*10000+MOD(B267,10)*1000+INT(MOD(B267,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="268" ht="20" customHeight="1">
+      <c r="A268" s="27" t="n">
+        <v>44189</v>
+      </c>
+      <c r="B268" s="28" t="n">
+        <v>59658</v>
+      </c>
+      <c r="C268" s="28">
+        <f>MOD(B268,100)*1000+INT(B268/100)</f>
+        <v/>
+      </c>
+      <c r="D268" s="28">
+        <f>INT(B268/10000)*10000+MOD(B268,10)*1000+INT(MOD(B268,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="269" ht="20" customHeight="1">
+      <c r="A269" s="29" t="n">
+        <v>44190</v>
+      </c>
+      <c r="B269" s="30" t="n">
+        <v>87577</v>
+      </c>
+      <c r="C269" s="30">
+        <f>MOD(B269,100)*1000+INT(B269/100)</f>
+        <v/>
+      </c>
+      <c r="D269" s="30">
+        <f>INT(B269/10000)*10000+MOD(B269,10)*1000+INT(MOD(B269,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="270" ht="20" customHeight="1">
+      <c r="A270" s="27" t="n">
+        <v>44191</v>
+      </c>
+      <c r="B270" s="28" t="n">
+        <v>96164</v>
+      </c>
+      <c r="C270" s="28">
+        <f>MOD(B270,100)*1000+INT(B270/100)</f>
+        <v/>
+      </c>
+      <c r="D270" s="28">
+        <f>INT(B270/10000)*10000+MOD(B270,10)*1000+INT(MOD(B270,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="271" ht="20" customHeight="1">
+      <c r="A271" s="29" t="n">
+        <v>44192</v>
+      </c>
+      <c r="B271" s="30" t="n">
+        <v>88062</v>
+      </c>
+      <c r="C271" s="30">
+        <f>MOD(B271,100)*1000+INT(B271/100)</f>
+        <v/>
+      </c>
+      <c r="D271" s="30">
+        <f>INT(B271/10000)*10000+MOD(B271,10)*1000+INT(MOD(B271,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="272" ht="20" customHeight="1">
+      <c r="A272" s="27" t="n">
+        <v>44193</v>
+      </c>
+      <c r="B272" s="28" t="n">
+        <v>26157</v>
+      </c>
+      <c r="C272" s="28">
+        <f>MOD(B272,100)*1000+INT(B272/100)</f>
+        <v/>
+      </c>
+      <c r="D272" s="28">
+        <f>INT(B272/10000)*10000+MOD(B272,10)*1000+INT(MOD(B272,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="273" ht="20" customHeight="1">
+      <c r="A273" s="29" t="n">
+        <v>44194</v>
+      </c>
+      <c r="B273" s="30" t="n">
+        <v>82743</v>
+      </c>
+      <c r="C273" s="30">
+        <f>MOD(B273,100)*1000+INT(B273/100)</f>
+        <v/>
+      </c>
+      <c r="D273" s="30">
+        <f>INT(B273/10000)*10000+MOD(B273,10)*1000+INT(MOD(B273,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="274" ht="20" customHeight="1">
+      <c r="A274" s="27" t="n">
+        <v>44195</v>
+      </c>
+      <c r="B274" s="28" t="n">
+        <v>27779</v>
+      </c>
+      <c r="C274" s="28">
+        <f>MOD(B274,100)*1000+INT(B274/100)</f>
+        <v/>
+      </c>
+      <c r="D274" s="28">
+        <f>INT(B274/10000)*10000+MOD(B274,10)*1000+INT(MOD(B274,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="275" ht="20" customHeight="1">
+      <c r="A275" s="29" t="n">
+        <v>44196</v>
+      </c>
+      <c r="B275" s="30" t="n">
+        <v>23846</v>
+      </c>
+      <c r="C275" s="30">
+        <f>MOD(B275,100)*1000+INT(B275/100)</f>
+        <v/>
+      </c>
+      <c r="D275" s="30">
+        <f>INT(B275/10000)*10000+MOD(B275,10)*1000+INT(MOD(B275,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="276" ht="20" customHeight="1">
+      <c r="A276" s="27" t="n">
+        <v>44197</v>
+      </c>
+      <c r="B276" s="28" t="n">
+        <v>29287</v>
+      </c>
+      <c r="C276" s="28">
+        <f>MOD(B276,100)*1000+INT(B276/100)</f>
+        <v/>
+      </c>
+      <c r="D276" s="28">
+        <f>INT(B276/10000)*10000+MOD(B276,10)*1000+INT(MOD(B276,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="277" ht="20" customHeight="1">
+      <c r="A277" s="29" t="n">
+        <v>44198</v>
+      </c>
+      <c r="B277" s="30" t="n">
+        <v>66010</v>
+      </c>
+      <c r="C277" s="30">
+        <f>MOD(B277,100)*1000+INT(B277/100)</f>
+        <v/>
+      </c>
+      <c r="D277" s="30">
+        <f>INT(B277/10000)*10000+MOD(B277,10)*1000+INT(MOD(B277,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="278" ht="20" customHeight="1">
+      <c r="A278" s="27" t="n">
+        <v>44199</v>
+      </c>
+      <c r="B278" s="28" t="n">
+        <v>47016</v>
+      </c>
+      <c r="C278" s="28">
+        <f>MOD(B278,100)*1000+INT(B278/100)</f>
+        <v/>
+      </c>
+      <c r="D278" s="28">
+        <f>INT(B278/10000)*10000+MOD(B278,10)*1000+INT(MOD(B278,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="279" ht="20" customHeight="1">
+      <c r="A279" s="29" t="n">
+        <v>44200</v>
+      </c>
+      <c r="B279" s="30" t="n">
+        <v>41083</v>
+      </c>
+      <c r="C279" s="30">
+        <f>MOD(B279,100)*1000+INT(B279/100)</f>
+        <v/>
+      </c>
+      <c r="D279" s="30">
+        <f>INT(B279/10000)*10000+MOD(B279,10)*1000+INT(MOD(B279,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="280" ht="20" customHeight="1">
+      <c r="A280" s="27" t="n">
+        <v>44201</v>
+      </c>
+      <c r="B280" s="28" t="n">
+        <v>16211</v>
+      </c>
+      <c r="C280" s="28">
+        <f>MOD(B280,100)*1000+INT(B280/100)</f>
+        <v/>
+      </c>
+      <c r="D280" s="28">
+        <f>INT(B280/10000)*10000+MOD(B280,10)*1000+INT(MOD(B280,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="281" ht="20" customHeight="1">
+      <c r="A281" s="29" t="n">
+        <v>44202</v>
+      </c>
+      <c r="B281" s="30" t="n">
+        <v>42890</v>
+      </c>
+      <c r="C281" s="30">
+        <f>MOD(B281,100)*1000+INT(B281/100)</f>
+        <v/>
+      </c>
+      <c r="D281" s="30">
+        <f>INT(B281/10000)*10000+MOD(B281,10)*1000+INT(MOD(B281,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="282" ht="20" customHeight="1">
+      <c r="A282" s="27" t="n">
+        <v>44203</v>
+      </c>
+      <c r="B282" s="28" t="n">
+        <v>83471</v>
+      </c>
+      <c r="C282" s="28">
+        <f>MOD(B282,100)*1000+INT(B282/100)</f>
+        <v/>
+      </c>
+      <c r="D282" s="28">
+        <f>INT(B282/10000)*10000+MOD(B282,10)*1000+INT(MOD(B282,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="283" ht="20" customHeight="1">
+      <c r="A283" s="29" t="n">
+        <v>44204</v>
+      </c>
+      <c r="B283" s="30" t="n">
+        <v>93502</v>
+      </c>
+      <c r="C283" s="30">
+        <f>MOD(B283,100)*1000+INT(B283/100)</f>
+        <v/>
+      </c>
+      <c r="D283" s="30">
+        <f>INT(B283/10000)*10000+MOD(B283,10)*1000+INT(MOD(B283,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="284" ht="20" customHeight="1">
+      <c r="A284" s="27" t="n">
+        <v>44205</v>
+      </c>
+      <c r="B284" s="28" t="n">
+        <v>64271</v>
+      </c>
+      <c r="C284" s="28">
+        <f>MOD(B284,100)*1000+INT(B284/100)</f>
+        <v/>
+      </c>
+      <c r="D284" s="28">
+        <f>INT(B284/10000)*10000+MOD(B284,10)*1000+INT(MOD(B284,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="285" ht="20" customHeight="1">
+      <c r="A285" s="29" t="n">
+        <v>44206</v>
+      </c>
+      <c r="B285" s="30" t="n">
+        <v>87288</v>
+      </c>
+      <c r="C285" s="30">
+        <f>MOD(B285,100)*1000+INT(B285/100)</f>
+        <v/>
+      </c>
+      <c r="D285" s="30">
+        <f>INT(B285/10000)*10000+MOD(B285,10)*1000+INT(MOD(B285,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="286" ht="20" customHeight="1">
+      <c r="A286" s="27" t="n">
+        <v>44207</v>
+      </c>
+      <c r="B286" s="28" t="n">
+        <v>22763</v>
+      </c>
+      <c r="C286" s="28">
+        <f>MOD(B286,100)*1000+INT(B286/100)</f>
+        <v/>
+      </c>
+      <c r="D286" s="28">
+        <f>INT(B286/10000)*10000+MOD(B286,10)*1000+INT(MOD(B286,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="287" ht="20" customHeight="1">
+      <c r="A287" s="29" t="n">
+        <v>44208</v>
+      </c>
+      <c r="B287" s="30" t="n">
+        <v>56150</v>
+      </c>
+      <c r="C287" s="30">
+        <f>MOD(B287,100)*1000+INT(B287/100)</f>
+        <v/>
+      </c>
+      <c r="D287" s="30">
+        <f>INT(B287/10000)*10000+MOD(B287,10)*1000+INT(MOD(B287,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="288" ht="20" customHeight="1">
+      <c r="A288" s="27" t="n">
+        <v>44209</v>
+      </c>
+      <c r="B288" s="28" t="n">
+        <v>60431</v>
+      </c>
+      <c r="C288" s="28">
+        <f>MOD(B288,100)*1000+INT(B288/100)</f>
+        <v/>
+      </c>
+      <c r="D288" s="28">
+        <f>INT(B288/10000)*10000+MOD(B288,10)*1000+INT(MOD(B288,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="289" ht="20" customHeight="1">
+      <c r="A289" s="29" t="n">
+        <v>44210</v>
+      </c>
+      <c r="B289" s="30" t="n">
+        <v>83622</v>
+      </c>
+      <c r="C289" s="30">
+        <f>MOD(B289,100)*1000+INT(B289/100)</f>
+        <v/>
+      </c>
+      <c r="D289" s="30">
+        <f>INT(B289/10000)*10000+MOD(B289,10)*1000+INT(MOD(B289,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="290" ht="20" customHeight="1">
+      <c r="A290" s="27" t="n">
+        <v>44211</v>
+      </c>
+      <c r="B290" s="28" t="n">
+        <v>22137</v>
+      </c>
+      <c r="C290" s="28">
+        <f>MOD(B290,100)*1000+INT(B290/100)</f>
+        <v/>
+      </c>
+      <c r="D290" s="28">
+        <f>INT(B290/10000)*10000+MOD(B290,10)*1000+INT(MOD(B290,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="291" ht="20" customHeight="1">
+      <c r="A291" s="29" t="n">
+        <v>44212</v>
+      </c>
+      <c r="B291" s="30" t="n">
+        <v>98095</v>
+      </c>
+      <c r="C291" s="30">
+        <f>MOD(B291,100)*1000+INT(B291/100)</f>
+        <v/>
+      </c>
+      <c r="D291" s="30">
+        <f>INT(B291/10000)*10000+MOD(B291,10)*1000+INT(MOD(B291,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="292" ht="20" customHeight="1">
+      <c r="A292" s="27" t="n">
+        <v>44213</v>
+      </c>
+      <c r="B292" s="28" t="n">
+        <v>87168</v>
+      </c>
+      <c r="C292" s="28">
+        <f>MOD(B292,100)*1000+INT(B292/100)</f>
+        <v/>
+      </c>
+      <c r="D292" s="28">
+        <f>INT(B292/10000)*10000+MOD(B292,10)*1000+INT(MOD(B292,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="293" ht="20" customHeight="1">
+      <c r="A293" s="29" t="n">
+        <v>44214</v>
+      </c>
+      <c r="B293" s="30" t="n">
+        <v>95667</v>
+      </c>
+      <c r="C293" s="30">
+        <f>MOD(B293,100)*1000+INT(B293/100)</f>
+        <v/>
+      </c>
+      <c r="D293" s="30">
+        <f>INT(B293/10000)*10000+MOD(B293,10)*1000+INT(MOD(B293,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="294" ht="20" customHeight="1">
+      <c r="A294" s="27" t="n">
+        <v>44215</v>
+      </c>
+      <c r="B294" s="28" t="n">
+        <v>28839</v>
+      </c>
+      <c r="C294" s="28">
+        <f>MOD(B294,100)*1000+INT(B294/100)</f>
+        <v/>
+      </c>
+      <c r="D294" s="28">
+        <f>INT(B294/10000)*10000+MOD(B294,10)*1000+INT(MOD(B294,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="295" ht="20" customHeight="1">
+      <c r="A295" s="29" t="n">
+        <v>44216</v>
+      </c>
+      <c r="B295" s="30" t="n">
+        <v>41618</v>
+      </c>
+      <c r="C295" s="30">
+        <f>MOD(B295,100)*1000+INT(B295/100)</f>
+        <v/>
+      </c>
+      <c r="D295" s="30">
+        <f>INT(B295/10000)*10000+MOD(B295,10)*1000+INT(MOD(B295,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="296" ht="20" customHeight="1">
+      <c r="A296" s="27" t="n">
+        <v>44217</v>
+      </c>
+      <c r="B296" s="28" t="n">
+        <v>58324</v>
+      </c>
+      <c r="C296" s="28">
+        <f>MOD(B296,100)*1000+INT(B296/100)</f>
+        <v/>
+      </c>
+      <c r="D296" s="28">
+        <f>INT(B296/10000)*10000+MOD(B296,10)*1000+INT(MOD(B296,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="297" ht="20" customHeight="1">
+      <c r="A297" s="29" t="n">
+        <v>44218</v>
+      </c>
+      <c r="B297" s="30" t="n">
+        <v>68394</v>
+      </c>
+      <c r="C297" s="30">
+        <f>MOD(B297,100)*1000+INT(B297/100)</f>
+        <v/>
+      </c>
+      <c r="D297" s="30">
+        <f>INT(B297/10000)*10000+MOD(B297,10)*1000+INT(MOD(B297,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="298" ht="20" customHeight="1">
+      <c r="A298" s="27" t="n">
+        <v>44219</v>
+      </c>
+      <c r="B298" s="28" t="n">
+        <v>68437</v>
+      </c>
+      <c r="C298" s="28">
+        <f>MOD(B298,100)*1000+INT(B298/100)</f>
+        <v/>
+      </c>
+      <c r="D298" s="28">
+        <f>INT(B298/10000)*10000+MOD(B298,10)*1000+INT(MOD(B298,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="299" ht="20" customHeight="1">
+      <c r="A299" s="29" t="n">
+        <v>44220</v>
+      </c>
+      <c r="B299" s="30" t="n">
+        <v>49390</v>
+      </c>
+      <c r="C299" s="30">
+        <f>MOD(B299,100)*1000+INT(B299/100)</f>
+        <v/>
+      </c>
+      <c r="D299" s="30">
+        <f>INT(B299/10000)*10000+MOD(B299,10)*1000+INT(MOD(B299,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="300" ht="20" customHeight="1">
+      <c r="A300" s="27" t="n">
+        <v>44221</v>
+      </c>
+      <c r="B300" s="28" t="n">
+        <v>28134</v>
+      </c>
+      <c r="C300" s="28">
+        <f>MOD(B300,100)*1000+INT(B300/100)</f>
+        <v/>
+      </c>
+      <c r="D300" s="28">
+        <f>INT(B300/10000)*10000+MOD(B300,10)*1000+INT(MOD(B300,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="301" ht="20" customHeight="1">
+      <c r="A301" s="29" t="n">
+        <v>44222</v>
+      </c>
+      <c r="B301" s="30" t="n">
+        <v>50283</v>
+      </c>
+      <c r="C301" s="30">
+        <f>MOD(B301,100)*1000+INT(B301/100)</f>
+        <v/>
+      </c>
+      <c r="D301" s="30">
+        <f>INT(B301/10000)*10000+MOD(B301,10)*1000+INT(MOD(B301,10000)/10)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D226"/>
+  <autoFilter ref="A1:D301"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>